<commit_message>
add performance timings to README.md file
</commit_message>
<xml_diff>
--- a/docs/Evaluation Question Manual Testing.xlsx
+++ b/docs/Evaluation Question Manual Testing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robkerr\projects\nfl-data-download\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3435094C-DE99-4CA4-B98D-28FA5D4CD283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0756044-E719-4CCF-9505-08152B288AC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34290" yWindow="1170" windowWidth="38620" windowHeight="21820" xr2:uid="{9F0101F7-F69D-41A6-809D-0EC8DCFBC855}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Question</t>
   </si>
@@ -117,6 +117,9 @@
   </si>
   <si>
     <t>Average</t>
+  </si>
+  <si>
+    <t>LH Advantage</t>
   </si>
 </sst>
 </file>
@@ -182,11 +185,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -199,12 +203,51 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="5">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -534,23 +577,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71FA1DCC-7B3B-4327-B7F9-CB26EE5E22B2}">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="84.5546875" customWidth="1"/>
     <col min="3" max="3" width="15.6640625" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="14.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
       <c r="B1" s="2"/>
       <c r="C1" s="3" t="s">
         <v>4</v>
       </c>
       <c r="D1" s="3"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1" s="7"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2" t="s">
         <v>0</v>
@@ -561,8 +606,11 @@
       <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E2" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -575,8 +623,12 @@
       <c r="D3">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E3" s="6">
+        <f>(C3-D3)/C3</f>
+        <v>0.45454545454545453</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -589,8 +641,12 @@
       <c r="D4">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E4" s="6">
+        <f t="shared" ref="E4:E23" si="0">(C4-D4)/C4</f>
+        <v>-0.2857142857142857</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
@@ -603,8 +659,12 @@
       <c r="D5">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E5" s="6">
+        <f t="shared" si="0"/>
+        <v>0.52173913043478259</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
@@ -617,8 +677,12 @@
       <c r="D6">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E6" s="6">
+        <f t="shared" si="0"/>
+        <v>0.41176470588235292</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>5</v>
       </c>
@@ -631,8 +695,12 @@
       <c r="D7">
         <v>9</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E7" s="6">
+        <f t="shared" si="0"/>
+        <v>0.35714285714285715</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
@@ -645,8 +713,12 @@
       <c r="D8">
         <v>11</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E8" s="6">
+        <f t="shared" si="0"/>
+        <v>0.57692307692307687</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>7</v>
       </c>
@@ -659,8 +731,12 @@
       <c r="D9">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E9" s="6">
+        <f t="shared" si="0"/>
+        <v>0.61904761904761907</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8</v>
       </c>
@@ -673,8 +749,12 @@
       <c r="D10">
         <v>10</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E10" s="6">
+        <f t="shared" si="0"/>
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>9</v>
       </c>
@@ -687,8 +767,12 @@
       <c r="D11">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E11" s="6">
+        <f t="shared" si="0"/>
+        <v>9.0909090909090912E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>10</v>
       </c>
@@ -701,8 +785,12 @@
       <c r="D12">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E12" s="6">
+        <f t="shared" si="0"/>
+        <v>0.16666666666666666</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>11</v>
       </c>
@@ -715,8 +803,12 @@
       <c r="D13">
         <v>8</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E13" s="6">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>12</v>
       </c>
@@ -729,8 +821,12 @@
       <c r="D14">
         <v>12</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E14" s="6">
+        <f t="shared" si="0"/>
+        <v>0.42857142857142855</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>13</v>
       </c>
@@ -743,10 +839,14 @@
       <c r="D15">
         <v>8</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E15" s="6">
+        <f t="shared" si="0"/>
+        <v>0.65217391304347827</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>11</v>
@@ -757,10 +857,14 @@
       <c r="D16">
         <v>10</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E16" s="6">
+        <f t="shared" si="0"/>
+        <v>0.52380952380952384</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>18</v>
@@ -771,10 +875,14 @@
       <c r="D17">
         <v>12</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E17" s="6">
+        <f t="shared" si="0"/>
+        <v>0.42857142857142855</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>17</v>
@@ -785,10 +893,14 @@
       <c r="D18">
         <v>8</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E18" s="6">
+        <f t="shared" si="0"/>
+        <v>0.52941176470588236</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>12</v>
@@ -799,10 +911,14 @@
       <c r="D19">
         <v>8</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E19" s="6">
+        <f t="shared" si="0"/>
+        <v>0.42857142857142855</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>16</v>
@@ -813,10 +929,14 @@
       <c r="D20">
         <v>8</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E20" s="6">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>13</v>
@@ -827,10 +947,14 @@
       <c r="D21">
         <v>9</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E21" s="6">
+        <f t="shared" si="0"/>
+        <v>0.52631578947368418</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>15</v>
@@ -841,10 +965,14 @@
       <c r="D22">
         <v>8</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E22" s="6">
+        <f t="shared" si="0"/>
+        <v>0.42857142857142855</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>14</v>
@@ -855,8 +983,12 @@
       <c r="D23">
         <v>10</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E23" s="6">
+        <f t="shared" si="0"/>
+        <v>0.56521739130434778</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B25" s="4" t="s">
         <v>25</v>
       </c>
@@ -878,11 +1010,25 @@
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="FF63C384"/>
+        <color rgb="FF008AEF"/>
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
           <x14:id>{0B9FF524-8BF4-4E6F-B606-D2986A20B4EA}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D3:D23">
+    <cfRule type="dataBar" priority="4">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF008AEF"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{39B7A51E-3719-402C-8085-0621F4FA260E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -896,7 +1042,7 @@
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FF63C384"/>
+              <x14:borderColor rgb="FF008AEF"/>
               <x14:negativeFillColor rgb="FFFF0000"/>
               <x14:negativeBorderColor rgb="FFFF0000"/>
               <x14:axisColor rgb="FF000000"/>
@@ -904,8 +1050,27 @@
           </x14:cfRule>
           <xm:sqref>C3:D23</xm:sqref>
         </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{39B7A51E-3719-402C-8085-0621F4FA260E}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF008AEF"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D3:D23</xm:sqref>
+        </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{f42aa342-8706-4288-bd11-ebb85995028c}" enabled="1" method="Standard" siteId="{72f988bf-86f1-41af-91ab-2d7cd011db47}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
update notebook content & documentation md and excel files
</commit_message>
<xml_diff>
--- a/docs/Evaluation Question Manual Testing.xlsx
+++ b/docs/Evaluation Question Manual Testing.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robkerr\projects\nfl-data-download\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robkerr\projects\nflverse-fabric-reference-architecture\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0756044-E719-4CCF-9505-08152B288AC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ACFEC5F-E3B3-4CA1-9532-09A9B88943A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34290" yWindow="1170" windowWidth="38620" windowHeight="21820" xr2:uid="{9F0101F7-F69D-41A6-809D-0EC8DCFBC855}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>Question</t>
   </si>
@@ -117,9 +117,6 @@
   </si>
   <si>
     <t>Average</t>
-  </si>
-  <si>
-    <t>LH Advantage</t>
   </si>
 </sst>
 </file>
@@ -128,7 +125,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="168" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -185,69 +182,29 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -577,25 +534,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71FA1DCC-7B3B-4327-B7F9-CB26EE5E22B2}">
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="84.5546875" customWidth="1"/>
     <col min="3" max="3" width="15.6640625" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="14.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
       <c r="B1" s="2"/>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="3"/>
-      <c r="E1" s="7"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D1" s="5"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2" t="s">
         <v>0</v>
@@ -606,11 +561,8 @@
       <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -623,12 +575,8 @@
       <c r="D3">
         <v>12</v>
       </c>
-      <c r="E3" s="6">
-        <f>(C3-D3)/C3</f>
-        <v>0.45454545454545453</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -641,12 +589,8 @@
       <c r="D4">
         <v>9</v>
       </c>
-      <c r="E4" s="6">
-        <f t="shared" ref="E4:E23" si="0">(C4-D4)/C4</f>
-        <v>-0.2857142857142857</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
@@ -659,12 +603,8 @@
       <c r="D5">
         <v>11</v>
       </c>
-      <c r="E5" s="6">
-        <f t="shared" si="0"/>
-        <v>0.52173913043478259</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
@@ -677,12 +617,8 @@
       <c r="D6">
         <v>10</v>
       </c>
-      <c r="E6" s="6">
-        <f t="shared" si="0"/>
-        <v>0.41176470588235292</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>5</v>
       </c>
@@ -695,12 +631,8 @@
       <c r="D7">
         <v>9</v>
       </c>
-      <c r="E7" s="6">
-        <f t="shared" si="0"/>
-        <v>0.35714285714285715</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
@@ -713,12 +645,8 @@
       <c r="D8">
         <v>11</v>
       </c>
-      <c r="E8" s="6">
-        <f t="shared" si="0"/>
-        <v>0.57692307692307687</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>7</v>
       </c>
@@ -731,12 +659,8 @@
       <c r="D9">
         <v>8</v>
       </c>
-      <c r="E9" s="6">
-        <f t="shared" si="0"/>
-        <v>0.61904761904761907</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8</v>
       </c>
@@ -749,12 +673,8 @@
       <c r="D10">
         <v>10</v>
       </c>
-      <c r="E10" s="6">
-        <f t="shared" si="0"/>
-        <v>0.375</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>9</v>
       </c>
@@ -767,12 +687,8 @@
       <c r="D11">
         <v>10</v>
       </c>
-      <c r="E11" s="6">
-        <f t="shared" si="0"/>
-        <v>9.0909090909090912E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>10</v>
       </c>
@@ -785,12 +701,8 @@
       <c r="D12">
         <v>10</v>
       </c>
-      <c r="E12" s="6">
-        <f t="shared" si="0"/>
-        <v>0.16666666666666666</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>11</v>
       </c>
@@ -803,12 +715,8 @@
       <c r="D13">
         <v>8</v>
       </c>
-      <c r="E13" s="6">
-        <f t="shared" si="0"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>12</v>
       </c>
@@ -821,12 +729,8 @@
       <c r="D14">
         <v>12</v>
       </c>
-      <c r="E14" s="6">
-        <f t="shared" si="0"/>
-        <v>0.42857142857142855</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>13</v>
       </c>
@@ -839,12 +743,8 @@
       <c r="D15">
         <v>8</v>
       </c>
-      <c r="E15" s="6">
-        <f t="shared" si="0"/>
-        <v>0.65217391304347827</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>14</v>
       </c>
@@ -857,12 +757,8 @@
       <c r="D16">
         <v>10</v>
       </c>
-      <c r="E16" s="6">
-        <f t="shared" si="0"/>
-        <v>0.52380952380952384</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>15</v>
       </c>
@@ -875,12 +771,8 @@
       <c r="D17">
         <v>12</v>
       </c>
-      <c r="E17" s="6">
-        <f t="shared" si="0"/>
-        <v>0.42857142857142855</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>16</v>
       </c>
@@ -893,12 +785,8 @@
       <c r="D18">
         <v>8</v>
       </c>
-      <c r="E18" s="6">
-        <f t="shared" si="0"/>
-        <v>0.52941176470588236</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>17</v>
       </c>
@@ -911,12 +799,8 @@
       <c r="D19">
         <v>8</v>
       </c>
-      <c r="E19" s="6">
-        <f t="shared" si="0"/>
-        <v>0.42857142857142855</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>18</v>
       </c>
@@ -929,12 +813,8 @@
       <c r="D20">
         <v>8</v>
       </c>
-      <c r="E20" s="6">
-        <f t="shared" si="0"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>19</v>
       </c>
@@ -947,12 +827,8 @@
       <c r="D21">
         <v>9</v>
       </c>
-      <c r="E21" s="6">
-        <f t="shared" si="0"/>
-        <v>0.52631578947368418</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>20</v>
       </c>
@@ -965,12 +841,8 @@
       <c r="D22">
         <v>8</v>
       </c>
-      <c r="E22" s="6">
-        <f t="shared" si="0"/>
-        <v>0.42857142857142855</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>21</v>
       </c>
@@ -983,20 +855,16 @@
       <c r="D23">
         <v>10</v>
       </c>
-      <c r="E23" s="6">
-        <f t="shared" si="0"/>
-        <v>0.56521739130434778</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B25" s="4" t="s">
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B25" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C25" s="5">
+      <c r="C25" s="4">
         <f>AVERAGE(C3:C23)</f>
         <v>17.80952380952381</v>
       </c>
-      <c r="D25" s="5">
+      <c r="D25" s="4">
         <f>AVERAGE(D3:D23)</f>
         <v>9.5714285714285712</v>
       </c>

</xml_diff>

<commit_message>
Update timings output to include DAX/SQL query latency
</commit_message>
<xml_diff>
--- a/docs/Evaluation Question Manual Testing.xlsx
+++ b/docs/Evaluation Question Manual Testing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robkerr\projects\nflverse-fabric-reference-architecture\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ACFEC5F-E3B3-4CA1-9532-09A9B88943A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B364E7F9-AD96-4A7A-BA8E-A28A36C9D084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34290" yWindow="1170" windowWidth="38620" windowHeight="21820" xr2:uid="{9F0101F7-F69D-41A6-809D-0EC8DCFBC855}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>Question</t>
   </si>
@@ -53,9 +53,6 @@
     <t>For QBs in 2025 with at least 100 clean dropbacks and at least 15 QB-hit dropbacks, who had the largest EPA per dropback differential between clean and QB-hit plays?</t>
   </si>
   <si>
-    <t>Response Time (seconds)</t>
-  </si>
-  <si>
     <t>How many regular-season NFL games were played in 2025?</t>
   </si>
   <si>
@@ -117,15 +114,31 @@
   </si>
   <si>
     <t>Average</t>
+  </si>
+  <si>
+    <t>Query Runtime (sec)</t>
+  </si>
+  <si>
+    <t>DAX</t>
+  </si>
+  <si>
+    <t>SQL</t>
+  </si>
+  <si>
+    <t>Data Agent Response Time (Sec)</t>
+  </si>
+  <si>
+    <t>Median</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -186,7 +199,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -196,6 +209,12 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -215,6 +234,118 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>92808</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>151423</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>405423</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>117230</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A91F1DCF-48D5-FCC9-2EA2-CF6CFB1E2D68}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="703385" y="6247423"/>
+          <a:ext cx="6110653" cy="1265115"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>Methodology:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>1. Each question pasted into data agent after pressing "Clear Chat" -- each question is the 1st in the conversation</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>2. Data agent time is the "Response time" taken from the Data Agent output step.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>3. For DAX</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t> Query time: D</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>AX query copy/pasted into Power</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t> BI Explore/DAX Query window </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t>4. For SQL Query time: SQL query copy/pasted into SQL Analytics Endpoint query window</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -534,23 +665,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71FA1DCC-7B3B-4327-B7F9-CB26EE5E22B2}">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="84.5546875" customWidth="1"/>
     <col min="3" max="3" width="15.6640625" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="16.21875" customWidth="1"/>
+    <col min="6" max="6" width="14.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
       <c r="B1" s="2"/>
-      <c r="C1" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="5"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C1" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" s="9"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2" t="s">
         <v>0</v>
@@ -561,320 +698,488 @@
       <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E2" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="7">
         <v>22</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="7">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E3" s="6">
+        <v>0.74</v>
+      </c>
+      <c r="F3" s="6">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4">
+        <v>4</v>
+      </c>
+      <c r="C4" s="7">
         <v>7</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="7">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E4" s="6">
+        <v>1.75</v>
+      </c>
+      <c r="F4" s="6">
+        <v>1.41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5">
         <v>23</v>
       </c>
-      <c r="D5">
+      <c r="C5" s="7">
+        <v>23</v>
+      </c>
+      <c r="D5" s="7">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E5" s="6">
+        <v>0.54</v>
+      </c>
+      <c r="F5" s="6">
+        <v>1.17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6">
+        <v>22</v>
+      </c>
+      <c r="C6" s="7">
         <v>17</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="7">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E6" s="6">
+        <v>0.6</v>
+      </c>
+      <c r="F6" s="6">
+        <v>1.1499999999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7">
+        <v>5</v>
+      </c>
+      <c r="C7" s="7">
         <v>14</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="7">
         <v>9</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E7" s="6">
+        <v>1.4</v>
+      </c>
+      <c r="F7" s="6">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8">
+        <v>21</v>
+      </c>
+      <c r="C8" s="7">
         <v>26</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="7">
         <v>11</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E8" s="6">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="F8" s="6">
+        <v>1.06</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9">
+        <v>6</v>
+      </c>
+      <c r="C9" s="7">
         <v>21</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="7">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E9" s="6">
+        <v>1.4</v>
+      </c>
+      <c r="F9" s="6">
+        <v>1.07</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10">
+        <v>7</v>
+      </c>
+      <c r="C10" s="7">
         <v>16</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="7">
         <v>10</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E10" s="6">
+        <v>1.3</v>
+      </c>
+      <c r="F10" s="6">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11">
+        <v>8</v>
+      </c>
+      <c r="C11" s="7">
         <v>11</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="7">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E11" s="6">
+        <v>0.6</v>
+      </c>
+      <c r="F11" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>10</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12">
+        <v>20</v>
+      </c>
+      <c r="C12" s="7">
         <v>12</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="7">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E12" s="6">
+        <v>1.4</v>
+      </c>
+      <c r="F12" s="6">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13">
+        <v>9</v>
+      </c>
+      <c r="C13" s="7">
         <v>16</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="7">
         <v>8</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E13" s="6">
+        <v>1.2</v>
+      </c>
+      <c r="F13" s="6">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C14">
+        <v>19</v>
+      </c>
+      <c r="C14" s="7">
         <v>21</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="7">
         <v>12</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E14" s="6">
+        <v>0.7</v>
+      </c>
+      <c r="F14" s="6">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15">
+        <v>18</v>
+      </c>
+      <c r="C15" s="7">
         <v>23</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="7">
         <v>8</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E15" s="6">
+        <v>0.6</v>
+      </c>
+      <c r="F15" s="6">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C16">
+        <v>10</v>
+      </c>
+      <c r="C16" s="7">
         <v>21</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="7">
         <v>10</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E16" s="6">
+        <v>1</v>
+      </c>
+      <c r="F16" s="6">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C17">
+        <v>17</v>
+      </c>
+      <c r="C17" s="7">
         <v>21</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="7">
         <v>12</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E17" s="6">
+        <v>0.7</v>
+      </c>
+      <c r="F17" s="6">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>16</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="7">
         <v>17</v>
       </c>
-      <c r="C18">
-        <v>17</v>
-      </c>
-      <c r="D18">
+      <c r="D18" s="7">
         <v>8</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E18" s="6">
+        <v>0.7</v>
+      </c>
+      <c r="F18" s="6">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>17</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C19">
+        <v>11</v>
+      </c>
+      <c r="C19" s="7">
         <v>14</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="7">
         <v>8</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E19" s="6">
+        <v>0.6</v>
+      </c>
+      <c r="F19" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>18</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" s="7">
         <v>16</v>
       </c>
-      <c r="C20">
-        <v>16</v>
-      </c>
-      <c r="D20">
+      <c r="D20" s="7">
         <v>8</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E20" s="6">
+        <v>1.6</v>
+      </c>
+      <c r="F20" s="6">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C21">
+        <v>12</v>
+      </c>
+      <c r="C21" s="7">
         <v>19</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="7">
         <v>9</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E21" s="6">
+        <v>0.7</v>
+      </c>
+      <c r="F21" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>20</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C22">
         <v>14</v>
       </c>
-      <c r="D22">
+      <c r="C22" s="7">
+        <v>14</v>
+      </c>
+      <c r="D22" s="7">
         <v>8</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E22" s="6">
+        <v>0.7</v>
+      </c>
+      <c r="F22" s="6">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>21</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C23">
+        <v>13</v>
+      </c>
+      <c r="C23" s="7">
         <v>23</v>
       </c>
-      <c r="D23">
+      <c r="D23" s="7">
         <v>10</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E23" s="6">
+        <v>0.9</v>
+      </c>
+      <c r="F23" s="6">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B25" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C25" s="4">
+        <v>24</v>
+      </c>
+      <c r="C25" s="8">
         <f>AVERAGE(C3:C23)</f>
         <v>17.80952380952381</v>
       </c>
-      <c r="D25" s="4">
+      <c r="D25" s="8">
         <f>AVERAGE(D3:D23)</f>
         <v>9.5714285714285712</v>
       </c>
+      <c r="E25" s="4">
+        <f t="shared" ref="E25:F25" si="0">AVERAGE(E3:E23)</f>
+        <v>0.96333333333333315</v>
+      </c>
+      <c r="F25" s="4">
+        <f t="shared" si="0"/>
+        <v>1.1042857142857141</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B26" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C26" s="8">
+        <f>MEDIAN(C3:C23)</f>
+        <v>17</v>
+      </c>
+      <c r="D26" s="8">
+        <f t="shared" ref="D26:F26" si="1">MEDIAN(D3:D23)</f>
+        <v>10</v>
+      </c>
+      <c r="E26" s="4">
+        <f t="shared" si="1"/>
+        <v>0.74</v>
+      </c>
+      <c r="F26" s="4">
+        <f t="shared" si="1"/>
+        <v>1.1000000000000001</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="C1:D1"/>
+    <mergeCell ref="E1:F1"/>
   </mergeCells>
-  <conditionalFormatting sqref="C3:D23">
-    <cfRule type="dataBar" priority="1">
+  <conditionalFormatting sqref="C3:D23 E4:F4 E3 E5:E23 F17:F23 F11:F13">
+    <cfRule type="dataBar" priority="2">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -887,8 +1192,8 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D3:D23">
-    <cfRule type="dataBar" priority="4">
+  <conditionalFormatting sqref="D3:D23 E4:F4 E3 E5:E23 F17:F23 F11:F13">
+    <cfRule type="dataBar" priority="5">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -901,7 +1206,22 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="E3:F23">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63C384"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{D853577E-7161-4E96-8DE3-B1C5C6CCB8D9}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -916,7 +1236,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C3:D23</xm:sqref>
+          <xm:sqref>C3:D23 E4:F4 E3 E5:E23 F17:F23 F11:F13</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{39B7A51E-3719-402C-8085-0621F4FA260E}">
@@ -929,7 +1249,20 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>D3:D23</xm:sqref>
+          <xm:sqref>D3:D23 E4:F4 E3 E5:E23 F17:F23 F11:F13</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{D853577E-7161-4E96-8DE3-B1C5C6CCB8D9}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF63C384"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E3:F23</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>

<commit_message>
Added median to timings report
</commit_message>
<xml_diff>
--- a/docs/Evaluation Question Manual Testing.xlsx
+++ b/docs/Evaluation Question Manual Testing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robkerr\projects\nflverse-fabric-reference-architecture\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B364E7F9-AD96-4A7A-BA8E-A28A36C9D084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09708E52-BC2C-4364-8D34-CBFC934B6EAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34290" yWindow="1170" windowWidth="38620" windowHeight="21820" xr2:uid="{9F0101F7-F69D-41A6-809D-0EC8DCFBC855}"/>
   </bookViews>
@@ -199,7 +199,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -208,16 +208,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -242,13 +241,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>92808</xdr:colOff>
-      <xdr:row>27</xdr:row>
+      <xdr:row>28</xdr:row>
       <xdr:rowOff>151423</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>405423</xdr:colOff>
-      <xdr:row>34</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>117230</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -678,14 +677,14 @@
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
       <c r="B1" s="2"/>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9" t="s">
+      <c r="D1" s="7"/>
+      <c r="E1" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="F1" s="9"/>
+      <c r="F1" s="7"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
@@ -698,10 +697,10 @@
       <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="4" t="s">
         <v>27</v>
       </c>
     </row>
@@ -712,16 +711,16 @@
       <c r="B3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="6">
         <v>22</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="6">
         <v>12</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="5">
         <v>0.74</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3" s="5">
         <v>0.78</v>
       </c>
     </row>
@@ -732,16 +731,16 @@
       <c r="B4" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="6">
         <v>7</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="6">
         <v>9</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="5">
         <v>1.75</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="5">
         <v>1.41</v>
       </c>
     </row>
@@ -752,16 +751,16 @@
       <c r="B5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="6">
         <v>23</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="6">
         <v>11</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="5">
         <v>0.54</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="5">
         <v>1.17</v>
       </c>
     </row>
@@ -772,16 +771,16 @@
       <c r="B6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="6">
         <v>17</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="6">
         <v>10</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="5">
         <v>0.6</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="5">
         <v>1.1499999999999999</v>
       </c>
     </row>
@@ -792,16 +791,16 @@
       <c r="B7" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="6">
         <v>14</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="6">
         <v>9</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="5">
         <v>1.4</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="5">
         <v>0.75</v>
       </c>
     </row>
@@ -812,16 +811,16 @@
       <c r="B8" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="6">
         <v>26</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="6">
         <v>11</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="5">
         <v>1.1000000000000001</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="5">
         <v>1.06</v>
       </c>
     </row>
@@ -832,16 +831,16 @@
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="6">
         <v>21</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="6">
         <v>8</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="5">
         <v>1.4</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="5">
         <v>1.07</v>
       </c>
     </row>
@@ -852,16 +851,16 @@
       <c r="B10" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="7">
+      <c r="C10" s="6">
         <v>16</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="6">
         <v>10</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="5">
         <v>1.3</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="5">
         <v>1.2</v>
       </c>
     </row>
@@ -872,16 +871,16 @@
       <c r="B11" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="6">
         <v>11</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="6">
         <v>10</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="5">
         <v>0.6</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="5">
         <v>1</v>
       </c>
     </row>
@@ -892,16 +891,16 @@
       <c r="B12" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="7">
+      <c r="C12" s="6">
         <v>12</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="6">
         <v>10</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="5">
         <v>1.4</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="5">
         <v>1.1000000000000001</v>
       </c>
     </row>
@@ -912,16 +911,16 @@
       <c r="B13" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="6">
         <v>16</v>
       </c>
-      <c r="D13" s="7">
+      <c r="D13" s="6">
         <v>8</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="5">
         <v>1.2</v>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="5">
         <v>1.1000000000000001</v>
       </c>
     </row>
@@ -932,16 +931,16 @@
       <c r="B14" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="7">
+      <c r="C14" s="6">
         <v>21</v>
       </c>
-      <c r="D14" s="7">
+      <c r="D14" s="6">
         <v>12</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="5">
         <v>0.7</v>
       </c>
-      <c r="F14" s="6">
+      <c r="F14" s="5">
         <v>1.1000000000000001</v>
       </c>
     </row>
@@ -952,16 +951,16 @@
       <c r="B15" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="7">
+      <c r="C15" s="6">
         <v>23</v>
       </c>
-      <c r="D15" s="7">
+      <c r="D15" s="6">
         <v>8</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="5">
         <v>0.6</v>
       </c>
-      <c r="F15" s="6">
+      <c r="F15" s="5">
         <v>1.2</v>
       </c>
     </row>
@@ -972,16 +971,16 @@
       <c r="B16" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="7">
+      <c r="C16" s="6">
         <v>21</v>
       </c>
-      <c r="D16" s="7">
+      <c r="D16" s="6">
         <v>10</v>
       </c>
-      <c r="E16" s="6">
+      <c r="E16" s="5">
         <v>1</v>
       </c>
-      <c r="F16" s="6">
+      <c r="F16" s="5">
         <v>1.2</v>
       </c>
     </row>
@@ -992,16 +991,16 @@
       <c r="B17" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="7">
+      <c r="C17" s="6">
         <v>21</v>
       </c>
-      <c r="D17" s="7">
+      <c r="D17" s="6">
         <v>12</v>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="5">
         <v>0.7</v>
       </c>
-      <c r="F17" s="6">
+      <c r="F17" s="5">
         <v>1.2</v>
       </c>
     </row>
@@ -1012,16 +1011,16 @@
       <c r="B18" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="7">
+      <c r="C18" s="6">
         <v>17</v>
       </c>
-      <c r="D18" s="7">
+      <c r="D18" s="6">
         <v>8</v>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="5">
         <v>0.7</v>
       </c>
-      <c r="F18" s="6">
+      <c r="F18" s="5">
         <v>1.2</v>
       </c>
     </row>
@@ -1032,16 +1031,16 @@
       <c r="B19" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C19" s="7">
+      <c r="C19" s="6">
         <v>14</v>
       </c>
-      <c r="D19" s="7">
+      <c r="D19" s="6">
         <v>8</v>
       </c>
-      <c r="E19" s="6">
+      <c r="E19" s="5">
         <v>0.6</v>
       </c>
-      <c r="F19" s="6">
+      <c r="F19" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1052,16 +1051,16 @@
       <c r="B20" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="7">
+      <c r="C20" s="6">
         <v>16</v>
       </c>
-      <c r="D20" s="7">
+      <c r="D20" s="6">
         <v>8</v>
       </c>
-      <c r="E20" s="6">
+      <c r="E20" s="5">
         <v>1.6</v>
       </c>
-      <c r="F20" s="6">
+      <c r="F20" s="5">
         <v>1.2</v>
       </c>
     </row>
@@ -1072,16 +1071,16 @@
       <c r="B21" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C21" s="7">
+      <c r="C21" s="6">
         <v>19</v>
       </c>
-      <c r="D21" s="7">
+      <c r="D21" s="6">
         <v>9</v>
       </c>
-      <c r="E21" s="6">
+      <c r="E21" s="5">
         <v>0.7</v>
       </c>
-      <c r="F21" s="6">
+      <c r="F21" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1092,16 +1091,16 @@
       <c r="B22" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C22" s="7">
+      <c r="C22" s="6">
         <v>14</v>
       </c>
-      <c r="D22" s="7">
+      <c r="D22" s="6">
         <v>8</v>
       </c>
-      <c r="E22" s="6">
+      <c r="E22" s="5">
         <v>0.7</v>
       </c>
-      <c r="F22" s="6">
+      <c r="F22" s="5">
         <v>1.1000000000000001</v>
       </c>
     </row>
@@ -1112,65 +1111,65 @@
       <c r="B23" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="7">
+      <c r="C23" s="6">
         <v>23</v>
       </c>
-      <c r="D23" s="7">
+      <c r="D23" s="6">
         <v>10</v>
       </c>
-      <c r="E23" s="6">
+      <c r="E23" s="5">
         <v>0.9</v>
       </c>
-      <c r="F23" s="6">
+      <c r="F23" s="5">
         <v>1.2</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B25" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25" s="8">
+        <f>MEDIAN(C3:C23)</f>
+        <v>17</v>
+      </c>
+      <c r="D25" s="8">
+        <f>MEDIAN(D3:D23)</f>
+        <v>10</v>
+      </c>
+      <c r="E25" s="8">
+        <f>MEDIAN(E3:E23)</f>
+        <v>0.74</v>
+      </c>
+      <c r="F25" s="8">
+        <f>MEDIAN(F3:F23)</f>
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B26" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C25" s="8">
+      <c r="C26" s="8">
         <f>AVERAGE(C3:C23)</f>
         <v>17.80952380952381</v>
       </c>
-      <c r="D25" s="8">
+      <c r="D26" s="8">
         <f>AVERAGE(D3:D23)</f>
         <v>9.5714285714285712</v>
       </c>
-      <c r="E25" s="4">
-        <f t="shared" ref="E25:F25" si="0">AVERAGE(E3:E23)</f>
+      <c r="E26" s="8">
+        <f t="shared" ref="E26:F26" si="0">AVERAGE(E3:E23)</f>
         <v>0.96333333333333315</v>
       </c>
-      <c r="F25" s="4">
+      <c r="F26" s="8">
         <f t="shared" si="0"/>
         <v>1.1042857142857141</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B26" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C26" s="8">
-        <f>MEDIAN(C3:C23)</f>
-        <v>17</v>
-      </c>
-      <c r="D26" s="8">
-        <f t="shared" ref="D26:F26" si="1">MEDIAN(D3:D23)</f>
-        <v>10</v>
-      </c>
-      <c r="E26" s="4">
-        <f t="shared" si="1"/>
-        <v>0.74</v>
-      </c>
-      <c r="F26" s="4">
-        <f t="shared" si="1"/>
-        <v>1.1000000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update testing excel file
</commit_message>
<xml_diff>
--- a/docs/Evaluation Question Manual Testing.xlsx
+++ b/docs/Evaluation Question Manual Testing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robkerr\projects\nflverse-fabric-reference-architecture\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09708E52-BC2C-4364-8D34-CBFC934B6EAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D3E36B9-62D0-4530-BBFE-375E72274F02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34290" yWindow="1170" windowWidth="38620" windowHeight="21820" xr2:uid="{9F0101F7-F69D-41A6-809D-0EC8DCFBC855}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{9F0101F7-F69D-41A6-809D-0EC8DCFBC855}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -172,7 +172,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -185,8 +185,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -194,12 +206,29 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -213,12 +242,17 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="4">
+    <cellStyle name="40% - Accent6" xfId="3" builtinId="51"/>
+    <cellStyle name="60% - Accent4" xfId="2" builtinId="44"/>
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -239,16 +273,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>92808</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>151423</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>120517</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>338458</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>405423</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>117230</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>290411</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -263,8 +297,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="703385" y="6247423"/>
-          <a:ext cx="6110653" cy="1265115"/>
+          <a:off x="12485699" y="1245931"/>
+          <a:ext cx="5746883" cy="1226571"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -667,8 +701,9 @@
   <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="3.5546875" customWidth="1"/>
     <col min="2" max="2" width="84.5546875" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" customWidth="1"/>
+    <col min="3" max="3" width="18.77734375" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="16.21875" customWidth="1"/>
     <col min="6" max="6" width="14.5546875" customWidth="1"/>
@@ -677,14 +712,14 @@
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
       <c r="B1" s="2"/>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7" t="s">
+      <c r="D1" s="9"/>
+      <c r="E1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="F1" s="7"/>
+      <c r="F1" s="8"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
@@ -704,11 +739,11 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="6">
@@ -728,7 +763,7 @@
       <c r="A4">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="6">
@@ -788,7 +823,7 @@
       <c r="A7">
         <v>5</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="6">
@@ -1134,19 +1169,19 @@
       <c r="B25" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="8">
+      <c r="C25" s="7">
         <f>MEDIAN(C3:C23)</f>
         <v>17</v>
       </c>
-      <c r="D25" s="8">
+      <c r="D25" s="7">
         <f>MEDIAN(D3:D23)</f>
         <v>10</v>
       </c>
-      <c r="E25" s="8">
+      <c r="E25" s="7">
         <f>MEDIAN(E3:E23)</f>
         <v>0.74</v>
       </c>
-      <c r="F25" s="8">
+      <c r="F25" s="7">
         <f>MEDIAN(F3:F23)</f>
         <v>1.1000000000000001</v>
       </c>
@@ -1155,19 +1190,19 @@
       <c r="B26" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C26" s="8">
+      <c r="C26" s="7">
         <f>AVERAGE(C3:C23)</f>
         <v>17.80952380952381</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="7">
         <f>AVERAGE(D3:D23)</f>
         <v>9.5714285714285712</v>
       </c>
-      <c r="E26" s="8">
+      <c r="E26" s="7">
         <f t="shared" ref="E26:F26" si="0">AVERAGE(E3:E23)</f>
         <v>0.96333333333333315</v>
       </c>
-      <c r="F26" s="8">
+      <c r="F26" s="7">
         <f t="shared" si="0"/>
         <v>1.1042857142857141</v>
       </c>
@@ -1177,44 +1212,16 @@
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="E1:F1"/>
   </mergeCells>
-  <conditionalFormatting sqref="C3:D23 E4:F4 E3 E5:E23 F17:F23 F11:F13">
-    <cfRule type="dataBar" priority="2">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF008AEF"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0B9FF524-8BF4-4E6F-B606-D2986A20B4EA}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D3:D23 E4:F4 E3 E5:E23 F17:F23 F11:F13">
-    <cfRule type="dataBar" priority="5">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF008AEF"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{39B7A51E-3719-402C-8085-0621F4FA260E}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E3:F23">
+  <conditionalFormatting sqref="C3:F23">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="FF63C384"/>
+        <color rgb="FF638EC6"/>
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D853577E-7161-4E96-8DE3-B1C5C6CCB8D9}</x14:id>
+          <x14:id>{769BB525-D2C8-462E-875F-B726D905BB0A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -1225,43 +1232,17 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0B9FF524-8BF4-4E6F-B606-D2986A20B4EA}">
+          <x14:cfRule type="dataBar" id="{769BB525-D2C8-462E-875F-B726D905BB0A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FF008AEF"/>
+              <x14:borderColor rgb="FF638EC6"/>
               <x14:negativeFillColor rgb="FFFF0000"/>
               <x14:negativeBorderColor rgb="FFFF0000"/>
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C3:D23 E4:F4 E3 E5:E23 F17:F23 F11:F13</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{39B7A51E-3719-402C-8085-0621F4FA260E}">
-            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FF008AEF"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:negativeBorderColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D3:D23 E4:F4 E3 E5:E23 F17:F23 F11:F13</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D853577E-7161-4E96-8DE3-B1C5C6CCB8D9}">
-            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FF63C384"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:negativeBorderColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>E3:F23</xm:sqref>
+          <xm:sqref>C3:F23</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>